<commit_message>
Update weekly ranking [2026-06-17]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -41,6 +41,7 @@
     <sheet name="magapoke_2026-05-27" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="magapoke_2026-06-03" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="magapoke_2026-06-10" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="magapoke_2026-06-17" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18680,6 +18681,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ブルーロック</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>信じていた仲間達にダンジョン奥地で殺されかけたがギフト『無限ガチャ』でレベル9999の仲間達を手に入れて元パーティーメンバーと世界に復讐＆『ざまぁ！』します！</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ドラハチ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ギルティサークル</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>東京卍リベンジャーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ハナバス　苔石花江のバスケ論</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>島耕作</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>魔女と傭兵</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>魔術ギルド総帥～生まれ変わって今更やり直す2度目の学院生活～</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>黒猫と魔女の教室</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>愛妻の裏アカ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>転生したら第七王子だったので、気ままに魔術を極めます</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ガチアクタ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>十字架のろくにん</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>転生貴族、鑑定スキルで成り上がる～弱小領地を受け継いだので、優秀な人材を増やしていたら、最強領地になってた～</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>WIND BREAKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>異世界ウォーキング</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>K-9~警視庁公安部公安第9課異能対策係~</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>となりの黒川さん</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-06-24]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -42,6 +42,7 @@
     <sheet name="magapoke_2026-06-03" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="magapoke_2026-06-10" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="magapoke_2026-06-17" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="magapoke_2026-06-24" sheetId="36" state="visible" r:id="rId36"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18957,6 +18958,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ブルーロック</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>WIND BREAKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ガチアクタ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>信じていた仲間達にダンジョン奥地で殺されかけたがギフト『無限ガチャ』でレベル9999の仲間達を手に入れて元パーティーメンバーと世界に復讐＆『ざまぁ！』します！</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>東京卍リベンジャーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ギルティサークル</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>FAIRY TAIL 100 YEARS QUEST</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>島耕作</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ハナバス　苔石花江のバスケ論</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>イレギュラーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>転生したら第七王子だったので、気ままに魔術を極めます</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>魔女と傭兵</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ハードワーカー中田</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ドラハチ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>十字架のろくにん</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>愛妻の裏アカ</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>転生貴族、鑑定スキルで成り上がる～弱小領地を受け継いだので、優秀な人材を増やしていたら、最強領地になってた～</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>魔術ギルド総帥～生まれ変わって今更やり直す2度目の学院生活～</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>君が僕らを悪魔と呼んだ頃</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>異世界ウォーキング</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>グラぱらっ！</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-07-01]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -43,6 +43,7 @@
     <sheet name="magapoke_2026-06-10" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="magapoke_2026-06-17" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="magapoke_2026-06-24" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="magapoke_2026-07-01" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19234,6 +19235,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ブルーロック</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>WIND BREAKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ガチアクタ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ギルティサークル</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ドラハチ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>東京卍リベンジャーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ハナバス　苔石花江のバスケ論</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>イレギュラーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>島耕作</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>信じていた仲間達にダンジョン奥地で殺されかけたがギフト『無限ガチャ』でレベル9999の仲間達を手に入れて元パーティーメンバーと世界に復讐＆『ざまぁ！』します！</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ハードワーカー中田</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>黒猫と魔女の教室</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>転生貴族、鑑定スキルで成り上がる～弱小領地を受け継いだので、優秀な人材を増やしていたら、最強領地になってた～</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>十字架のろくにん</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>転生したら第七王子だったので、気ままに魔術を極めます</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>愛妻の裏アカ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>魔女と傭兵</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>となりの黒川さん</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>魔術ギルド総帥～生まれ変わって今更やり直す2度目の学院生活～</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>蒼く染めろ</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-07-08]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -44,6 +44,7 @@
     <sheet name="magapoke_2026-06-17" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="magapoke_2026-06-24" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="magapoke_2026-07-01" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="magapoke_2026-07-08" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19511,6 +19512,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ブルーロック</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>WIND BREAKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ガチアクタ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ギルティサークル</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>東京卍リベンジャーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>信じていた仲間達にダンジョン奥地で殺されかけたがギフト『無限ガチャ』でレベル9999の仲間達を手に入れて元パーティーメンバーと世界に復讐＆『ざまぁ！』します！</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ハナバス　苔石花江のバスケ論</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FAIRY TAIL 100 YEARS QUEST</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>イレギュラーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>転生したら第七王子だったので、気ままに魔術を極めます</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>島耕作</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>愛妻の裏アカ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>君が僕らを悪魔と呼んだ頃</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>魔女と傭兵</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ハードワーカー中田</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>十字架のろくにん</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>転生貴族、鑑定スキルで成り上がる～弱小領地を受け継いだので、優秀な人材を増やしていたら、最強領地になってた～</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>魔術ギルド総帥～生まれ変わって今更やり直す2度目の学院生活～</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>蒼く染めろ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ドラハチ</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-07-15]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -45,6 +45,7 @@
     <sheet name="magapoke_2026-06-24" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="magapoke_2026-07-01" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="magapoke_2026-07-08" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="magapoke_2026-07-15" sheetId="39" state="visible" r:id="rId39"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19788,6 +19789,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ブルーロック</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>WIND BREAKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>信じていた仲間達にダンジョン奥地で殺されかけたがギフト『無限ガチャ』でレベル9999の仲間達を手に入れて元パーティーメンバーと世界に復讐＆『ざまぁ！』します！</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>東京卍リベンジャーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ギルティサークル</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ハナバス　苔石花江のバスケ論</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ドラハチ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>島耕作</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>イレギュラーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>君が僕らを悪魔と呼んだ頃</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>愛妻の裏アカ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ハードワーカー中田</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>魔女と傭兵</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>黒猫と魔女の教室</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>十字架のろくにん</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ガチアクタ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>となりの黒川さん</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>転生貴族、鑑定スキルで成り上がる～弱小領地を受け継いだので、優秀な人材を増やしていたら、最強領地になってた～</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>転生したら第七王子だったので、気ままに魔術を極めます</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>異世界ウォーキング</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>魔術ギルド総帥～生まれ変わって今更やり直す2度目の学院生活～</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-07-22]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -46,6 +46,7 @@
     <sheet name="magapoke_2026-07-01" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="magapoke_2026-07-08" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="magapoke_2026-07-15" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="magapoke_2026-07-22" sheetId="40" state="visible" r:id="rId40"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21091,6 +21092,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>WIND BREAKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ブルーロック</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>信じていた仲間達にダンジョン奥地で殺されかけたがギフト『無限ガチャ』でレベル9999の仲間達を手に入れて元パーティーメンバーと世界に復讐＆『ざまぁ！』します！</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ハナバス　苔石花江のバスケ論</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ガチアクタ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ギルティサークル</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>東京卍リベンジャーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FAIRY TAIL 100 YEARS QUEST</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>島耕作</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>転生したら第七王子だったので、気ままに魔術を極めます</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>イレギュラーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>愛妻の裏アカ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>君が僕らを悪魔と呼んだ頃</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>魔女と傭兵</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ハードワーカー中田</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>十字架のろくにん</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>蒼く染めろ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ドラハチ</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>K-9~警視庁公安部公安第9課異能対策係~</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>魔術ギルド総帥～生まれ変わって今更やり直す2度目の学院生活～</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>異世界ウォーキング</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-07-29]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -47,6 +47,7 @@
     <sheet name="magapoke_2026-07-08" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="magapoke_2026-07-15" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="magapoke_2026-07-22" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="magapoke_2026-07-29" sheetId="41" state="visible" r:id="rId41"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21368,6 +21369,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ブルーロック</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>WIND BREAKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ガチアクタ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>東京卍リベンジャーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ハナバス　苔石花江のバスケ論</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>となりの黒川さん</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>島耕作</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>イレギュラーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>十字架のろくにん</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>信じていた仲間達にダンジョン奥地で殺されかけたがギフト『無限ガチャ』でレベル9999の仲間達を手に入れて元パーティーメンバーと世界に復讐＆『ざまぁ！』します！</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>黒猫と魔女の教室</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ギルティサークル</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>君が僕らを悪魔と呼んだ頃</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>魔術ギルド総帥～生まれ変わって今更やり直す2度目の学院生活～</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>蒼く染めろ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>魔女と傭兵</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>転生したら第七王子だったので、気ままに魔術を極めます</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>食糧人類-Starving Anonymous-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>K-9~警視庁公安部公安第9課異能対策係~</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-08-05]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -48,6 +48,7 @@
     <sheet name="magapoke_2026-07-15" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="magapoke_2026-07-22" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="magapoke_2026-07-29" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="magapoke_2026-08-05" sheetId="42" state="visible" r:id="rId42"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21645,6 +21646,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ブルーロック</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ガチアクタ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>信じていた仲間達にダンジョン奥地で殺されかけたがギフト『無限ガチャ』でレベル9999の仲間達を手に入れて元パーティーメンバーと世界に復讐＆『ざまぁ！』します！</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ハナバス　苔石花江のバスケ論</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>東京卍リベンジャーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ギルティサークル</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ドラハチ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FAIRY TAIL 100 YEARS QUEST</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>転生したら第七王子だったので、気ままに魔術を極めます</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>島耕作</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>イレギュラーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>君が僕らを悪魔と呼んだ頃</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>愛妻の裏アカ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>十字架のろくにん</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>魔女と傭兵</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ハードワーカー中田</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>食糧人類-Starving Anonymous-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>WIND BREAKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>蒼く染めろ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>転生貴族、鑑定スキルで成り上がる～弱小領地を受け継いだので、優秀な人材を増やしていたら、最強領地になってた～</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>魔術ギルド総帥～生まれ変わって今更やり直す2度目の学院生活～</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-08-12]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -49,6 +49,7 @@
     <sheet name="magapoke_2026-07-22" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="magapoke_2026-07-29" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="magapoke_2026-08-05" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="magapoke_2026-08-12" sheetId="43" state="visible" r:id="rId43"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21922,6 +21923,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ブルーロック</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>WIND BREAKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ハナバス　苔石花江のバスケ論</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>信じていた仲間達にダンジョン奥地で殺されかけたがギフト『無限ガチャ』でレベル9999の仲間達を手に入れて元パーティーメンバーと世界に復讐＆『ざまぁ！』します！</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ギルティサークル</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>東京卍リベンジャーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>島耕作</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>君が僕らを悪魔と呼んだ頃</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>イレギュラーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ヒトの心が読める彼女の話</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ハードワーカー中田</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>黒猫と魔女の教室</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>転生したら第七王子だったので、気ままに魔術を極めます</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>愛妻の裏アカ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>十字架のろくにん</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>異世界ウォーキング</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>蒼く染めろ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>となりの黒川さん</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>食糧人類-Starving Anonymous-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>魔術ギルド総帥～生まれ変わって今更やり直す2度目の学院生活～</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>K-9~警視庁公安部公安第9課異能対策係~</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-08-19]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -50,6 +50,7 @@
     <sheet name="magapoke_2026-07-29" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="magapoke_2026-08-05" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="magapoke_2026-08-12" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="magapoke_2026-08-19" sheetId="44" state="visible" r:id="rId44"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22199,6 +22200,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ブルーロック</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>信じていた仲間達にダンジョン奥地で殺されかけたがギフト『無限ガチャ』でレベル9999の仲間達を手に入れて元パーティーメンバーと世界に復讐＆『ざまぁ！』します！</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ハナバス　苔石花江のバスケ論</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>東京卍リベンジャーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ギルティサークル</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>FAIRY TAIL 100 YEARS QUEST</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ドラハチ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>島耕作</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>転生したら第七王子だったので、気ままに魔術を極めます</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>イレギュラーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>限界集落を脱村した錬金術士、都会で"最強"なのがバレまくる。～老害どもにはいい加減愛想が尽きました～</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>君が僕らを悪魔と呼んだ頃</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>魔女と傭兵</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>愛妻の裏アカ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ハードワーカー中田</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>異世界ウォーキング</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>蒼く染めろ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>十字架のろくにん</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>魔術ギルド総帥～生まれ変わって今更やり直す2度目の学院生活～</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>WIND BREAKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ガチアクタ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ヒトの心が読める彼女の話</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>